<commit_message>
Agents Report page and minor changes
</commit_message>
<xml_diff>
--- a/public/assets/TimesheetUpload.xlsx
+++ b/public/assets/TimesheetUpload.xlsx
@@ -5,15 +5,15 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hussain\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admibn\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F6A2F0CD-8D04-48E4-A139-D16AAB7D24F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBCBED4D-F6BE-4989-BEEE-3AF071E415E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9BF946EE-887E-4E6E-A9C1-132354D3825D}"/>
+    <workbookView xWindow="3420" yWindow="3420" windowWidth="21600" windowHeight="11385" xr2:uid="{9BF946EE-887E-4E6E-A9C1-132354D3825D}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="3" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
   <si>
     <t>AgentId</t>
   </si>
@@ -72,31 +72,25 @@
     <t>Saturday</t>
   </si>
   <si>
+    <t>Morning</t>
+  </si>
+  <si>
+    <t>BCT-BurhanJivanji</t>
+  </si>
+  <si>
+    <t>Burhan Jivanji</t>
+  </si>
+  <si>
+    <t>Deepak</t>
+  </si>
+  <si>
     <t>Abbas</t>
   </si>
   <si>
-    <t>Burhan</t>
-  </si>
-  <si>
-    <t>Deepak</t>
-  </si>
-  <si>
-    <t>Mahmoud</t>
-  </si>
-  <si>
-    <t>Ismail</t>
-  </si>
-  <si>
-    <t>Morning</t>
-  </si>
-  <si>
-    <t>Evening</t>
-  </si>
-  <si>
-    <t>Afternoon</t>
-  </si>
-  <si>
-    <t>Shenouda</t>
+    <t>BCT-DeepakNagda</t>
+  </si>
+  <si>
+    <t>BCT-AbbasBohra</t>
   </si>
 </sst>
 </file>
@@ -473,21 +467,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE4C0EB1-D617-498C-A869-EAD3E8C173D6}">
-  <dimension ref="A1:L11"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98B49181-B3BA-4EAE-AFFD-44FDD79250E1}">
+  <dimension ref="A1:L4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.7109375" customWidth="1"/>
+    <col min="2" max="2" width="13.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -529,20 +514,20 @@
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
-        <v>1</v>
+      <c r="A2" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>18</v>
-      </c>
       <c r="D2" s="2">
-        <v>0.41666666666666669</v>
+        <v>0.29166666666666669</v>
       </c>
       <c r="E2" s="2">
-        <v>0.49930555555555556</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="F2" s="1">
         <v>1</v>
@@ -554,33 +539,33 @@
         <v>1</v>
       </c>
       <c r="I2" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J2" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K2" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L2" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="1">
-        <v>1</v>
+      <c r="A3" s="1" t="s">
+        <v>17</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>17</v>
-      </c>
       <c r="D3" s="2">
-        <v>0</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="E3" s="2">
-        <v>0.16666666666666666</v>
+        <v>0.70833333333333337</v>
       </c>
       <c r="F3" s="1">
         <v>1</v>
@@ -605,20 +590,20 @@
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" s="1">
-        <v>2</v>
+      <c r="A4" s="1" t="s">
+        <v>18</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="D4" s="2">
-        <v>0.33333333333333331</v>
+        <v>0.375</v>
       </c>
       <c r="E4" s="2">
-        <v>0.66666666666666663</v>
+        <v>0.75</v>
       </c>
       <c r="F4" s="1">
         <v>1</v>
@@ -627,10 +612,10 @@
         <v>1</v>
       </c>
       <c r="H4" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I4" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" s="1">
         <v>0</v>
@@ -639,272 +624,6 @@
         <v>1</v>
       </c>
       <c r="L4" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
-        <v>3</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="2">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="E5" s="2">
-        <v>0.49930555555555556</v>
-      </c>
-      <c r="F5" s="1">
-        <v>1</v>
-      </c>
-      <c r="G5" s="1">
-        <v>1</v>
-      </c>
-      <c r="H5" s="1">
-        <v>0</v>
-      </c>
-      <c r="I5" s="1">
-        <v>1</v>
-      </c>
-      <c r="J5" s="1">
-        <v>1</v>
-      </c>
-      <c r="K5" s="1">
-        <v>1</v>
-      </c>
-      <c r="L5" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A6" s="1">
-        <v>3</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="2">
-        <v>0</v>
-      </c>
-      <c r="E6" s="2">
-        <v>0.16666666666666666</v>
-      </c>
-      <c r="F6" s="1">
-        <v>1</v>
-      </c>
-      <c r="G6" s="1">
-        <v>1</v>
-      </c>
-      <c r="H6" s="1">
-        <v>1</v>
-      </c>
-      <c r="I6" s="1">
-        <v>1</v>
-      </c>
-      <c r="J6" s="1">
-        <v>0</v>
-      </c>
-      <c r="K6" s="1">
-        <v>1</v>
-      </c>
-      <c r="L6" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A7" s="1">
-        <v>4</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="E7" s="2">
-        <v>0.66666666666666663</v>
-      </c>
-      <c r="F7" s="1">
-        <v>1</v>
-      </c>
-      <c r="G7" s="1">
-        <v>0</v>
-      </c>
-      <c r="H7" s="1">
-        <v>1</v>
-      </c>
-      <c r="I7" s="1">
-        <v>1</v>
-      </c>
-      <c r="J7" s="1">
-        <v>1</v>
-      </c>
-      <c r="K7" s="1">
-        <v>1</v>
-      </c>
-      <c r="L7" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A8" s="1">
-        <v>4</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D8" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="E8" s="2">
-        <v>0.70833333333333337</v>
-      </c>
-      <c r="F8" s="1">
-        <v>1</v>
-      </c>
-      <c r="G8" s="1">
-        <v>1</v>
-      </c>
-      <c r="H8" s="1">
-        <v>1</v>
-      </c>
-      <c r="I8" s="1">
-        <v>1</v>
-      </c>
-      <c r="J8" s="1">
-        <v>1</v>
-      </c>
-      <c r="K8" s="1">
-        <v>0</v>
-      </c>
-      <c r="L8" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A9" s="1">
-        <v>5</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D9" s="2">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="E9" s="2">
-        <v>0.49930555555555556</v>
-      </c>
-      <c r="F9" s="1">
-        <v>1</v>
-      </c>
-      <c r="G9" s="1">
-        <v>0</v>
-      </c>
-      <c r="H9" s="1">
-        <v>1</v>
-      </c>
-      <c r="I9" s="1">
-        <v>1</v>
-      </c>
-      <c r="J9" s="1">
-        <v>1</v>
-      </c>
-      <c r="K9" s="1">
-        <v>1</v>
-      </c>
-      <c r="L9" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A10" s="1">
-        <v>5</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D10" s="2">
-        <v>0</v>
-      </c>
-      <c r="E10" s="2">
-        <v>0.16666666666666666</v>
-      </c>
-      <c r="F10" s="1">
-        <v>1</v>
-      </c>
-      <c r="G10" s="1">
-        <v>1</v>
-      </c>
-      <c r="H10" s="1">
-        <v>1</v>
-      </c>
-      <c r="I10" s="1">
-        <v>1</v>
-      </c>
-      <c r="J10" s="1">
-        <v>1</v>
-      </c>
-      <c r="K10" s="1">
-        <v>0</v>
-      </c>
-      <c r="L10" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A11" s="1">
-        <v>6</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D11" s="2">
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="E11" s="2">
-        <v>0.66666666666666663</v>
-      </c>
-      <c r="F11" s="1">
-        <v>1</v>
-      </c>
-      <c r="G11" s="1">
-        <v>1</v>
-      </c>
-      <c r="H11" s="1">
-        <v>0</v>
-      </c>
-      <c r="I11" s="1">
-        <v>1</v>
-      </c>
-      <c r="J11" s="1">
-        <v>1</v>
-      </c>
-      <c r="K11" s="1">
-        <v>1</v>
-      </c>
-      <c r="L11" s="1">
         <v>1</v>
       </c>
     </row>

</xml_diff>